<commit_message>
Colonna Giocato: Edo e Nic in campo vs Trecate, Vala assente
</commit_message>
<xml_diff>
--- a/Turate/Turate_Basket.xlsx
+++ b/Turate/Turate_Basket.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="45">
   <si>
     <t xml:space="preserve">Partita</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t xml:space="preserve">Palle rubate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giocato</t>
   </si>
   <si>
     <t xml:space="preserve">Jack</t>
@@ -451,7 +454,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R66"/>
+  <dimension ref="A1:S66"/>
   <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -509,13 +512,16 @@
       <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="S1" s="0" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>1</v>
@@ -563,7 +569,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>1</v>
@@ -611,7 +617,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>1</v>
@@ -659,7 +665,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>1</v>
@@ -707,7 +713,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>1</v>
@@ -755,7 +761,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>0</v>
@@ -803,7 +809,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>0</v>
@@ -851,7 +857,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>0</v>
@@ -899,7 +905,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>0</v>
@@ -947,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>0</v>
@@ -995,7 +1001,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>0</v>
@@ -1043,7 +1049,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>0</v>
@@ -1091,7 +1097,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" s="1" t="n">
         <f aca="false">SUM(C2:C13)</f>
@@ -1147,7 +1153,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>1</v>
@@ -1195,7 +1201,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>1</v>
@@ -1243,7 +1249,7 @@
         <v>2</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="1" t="n">
         <v>1</v>
@@ -1291,7 +1297,7 @@
         <v>2</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
@@ -1339,7 +1345,7 @@
         <v>2</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
@@ -1387,7 +1393,7 @@
         <v>2</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>0</v>
@@ -1435,7 +1441,7 @@
         <v>2</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>0</v>
@@ -1483,7 +1489,7 @@
         <v>2</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>0</v>
@@ -1531,7 +1537,7 @@
         <v>2</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C23" s="1" t="n">
         <v>0</v>
@@ -1579,7 +1585,7 @@
         <v>2</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>0</v>
@@ -1627,7 +1633,7 @@
         <v>2</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>0</v>
@@ -1675,7 +1681,7 @@
         <v>2</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C26" s="1" t="n">
         <v>0</v>
@@ -1723,7 +1729,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C27" s="1" t="n">
         <f aca="false">SUM(C15:C26)</f>
@@ -1779,7 +1785,7 @@
         <v>3</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C28" s="1" t="n">
         <v>1</v>
@@ -1827,7 +1833,7 @@
         <v>3</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C29" s="1" t="n">
         <v>1</v>
@@ -1875,7 +1881,7 @@
         <v>3</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C30" s="1" t="n">
         <v>1</v>
@@ -1923,7 +1929,7 @@
         <v>3</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C31" s="1" t="n">
         <v>1</v>
@@ -1971,7 +1977,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C32" s="1" t="n">
         <v>1</v>
@@ -2019,7 +2025,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C33" s="1" t="n">
         <v>0</v>
@@ -2067,7 +2073,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C34" s="1" t="n">
         <v>0</v>
@@ -2115,7 +2121,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C35" s="1" t="n">
         <v>0</v>
@@ -2163,7 +2169,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C36" s="1" t="n">
         <v>0</v>
@@ -2211,7 +2217,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C37" s="1" t="n">
         <v>0</v>
@@ -2259,7 +2265,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C38" s="1" t="n">
         <v>0</v>
@@ -2307,7 +2313,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C39" s="1" t="n">
         <v>0</v>
@@ -2355,7 +2361,7 @@
         <v>3</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C40" s="1" t="n">
         <f aca="false">SUM(C28:C39)</f>
@@ -2411,7 +2417,7 @@
         <v>4</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C41" s="1" t="n">
         <v>1</v>
@@ -2471,7 +2477,7 @@
         <v>4</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C42" s="1" t="n">
         <v>1</v>
@@ -2531,7 +2537,7 @@
         <v>4</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C43" s="1" t="n">
         <v>1</v>
@@ -2591,7 +2597,7 @@
         <v>4</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C44" s="1" t="n">
         <v>0</v>
@@ -2651,7 +2657,7 @@
         <v>4</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C45" s="1" t="n">
         <v>1</v>
@@ -2711,7 +2717,7 @@
         <v>4</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C46" s="1" t="n">
         <v>0</v>
@@ -2771,7 +2777,7 @@
         <v>4</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C47" s="1" t="n">
         <v>0</v>
@@ -2831,7 +2837,7 @@
         <v>4</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C48" s="1" t="n">
         <v>0</v>
@@ -2891,7 +2897,7 @@
         <v>4</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C49" s="1" t="n">
         <v>0</v>
@@ -2951,7 +2957,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C50" s="1" t="n">
         <v>0</v>
@@ -3011,7 +3017,7 @@
         <v>4</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C51" s="1" t="n">
         <v>1</v>
@@ -3071,7 +3077,7 @@
         <v>4</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C52" s="1" t="n">
         <v>0</v>
@@ -3131,7 +3137,7 @@
         <v>4</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C53" s="1" t="n">
         <f aca="false">SUM(C41:C52)</f>
@@ -3203,7 +3209,7 @@
         <v>5</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C54" s="1" t="n">
         <v>1</v>
@@ -3257,13 +3263,16 @@
       <c r="R54" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="S54" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C55" s="1" t="n">
         <v>1</v>
@@ -3317,13 +3326,16 @@
       <c r="R55" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="S55" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C56" s="1" t="n">
         <v>1</v>
@@ -3377,13 +3389,16 @@
       <c r="R56" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="S56" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C57" s="1" t="n">
         <v>0</v>
@@ -3437,13 +3452,16 @@
       <c r="R57" s="1" t="n">
         <v>3</v>
       </c>
+      <c r="S57" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C58" s="1" t="n">
         <v>1</v>
@@ -3497,13 +3515,16 @@
       <c r="R58" s="1" t="n">
         <v>4</v>
       </c>
+      <c r="S58" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C59" s="1" t="n">
         <v>0</v>
@@ -3557,13 +3578,16 @@
       <c r="R59" s="1" t="n">
         <v>2</v>
       </c>
+      <c r="S59" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C60" s="1" t="n">
         <v>0</v>
@@ -3617,13 +3641,16 @@
       <c r="R60" s="1" t="n">
         <v>1</v>
       </c>
+      <c r="S60" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C61" s="1" t="n">
         <v>1</v>
@@ -3676,6 +3703,9 @@
       </c>
       <c r="R61" s="1" t="n">
         <v>2</v>
+      </c>
+      <c r="S61" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3683,7 +3713,7 @@
         <v>5</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C62" s="1" t="n">
         <v>0</v>
@@ -3736,6 +3766,9 @@
       </c>
       <c r="R62" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="S62" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3743,7 +3776,7 @@
         <v>5</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C63" s="1" t="n">
         <v>0</v>
@@ -3796,6 +3829,9 @@
       </c>
       <c r="R63" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="S63" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3803,7 +3839,7 @@
         <v>5</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C64" s="1" t="n">
         <v>0</v>
@@ -3855,6 +3891,9 @@
         <v>0</v>
       </c>
       <c r="R64" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="S64" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3863,7 +3902,7 @@
         <v>5</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C65" s="1" t="n">
         <v>0</v>
@@ -3916,6 +3955,9 @@
       </c>
       <c r="R65" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="S65" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3923,7 +3965,7 @@
         <v>5</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C66" s="1" t="n">
         <f aca="false">SUM(C54:C65)</f>
@@ -3988,6 +4030,10 @@
       <c r="R66" s="1" t="n">
         <f aca="false">SUM(R54:R65)</f>
         <v>16</v>
+      </c>
+      <c r="S66" s="0" t="n">
+        <f aca="false">SUM(S54:S65)</f>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4011,22 +4057,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4037,10 +4083,10 @@
         <v>46287</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>81</v>
@@ -4057,10 +4103,10 @@
         <v>46299</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>75</v>
@@ -4077,10 +4123,10 @@
         <v>46299</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>46</v>
@@ -4097,10 +4143,10 @@
         <v>46312</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>72</v>
@@ -4117,10 +4163,10 @@
         <v>46320</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>67</v>

</xml_diff>